<commit_message>
README and notes: tested on a second Mac (MacBook Air via Thunderbolt-to-FireWire adapter)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PROVENANCE-MATRIX.xlsx
+++ b/PROVENANCE-MATRIX.xlsx
@@ -27758,7 +27758,7 @@
       </c>
       <c r="I39" s="77" t="inlineStr">
         <is>
-          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: tests/hw-smoke/integrated.sh. Regra do avião: este é o ÚNICO teste de hardware integrado; sem testes parciais. [2026-10-16] Roteiro tests/hw-smoke/integrated.sh escrito (13 passos, --preflight rodado no build PC); falta a execução com você presente. [2026-10-16 1º teste integrado] Primeira execução feita (passos 0-6 parcialmente); kextunload causou panic (HSCI em voo, corrigido F10 no código). Ver build-pc-runs/2026-10-16-first-integrated-run.md.</t>
+          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: tests/hw-smoke/integrated.sh. Regra do avião: este é o ÚNICO teste de hardware integrado; sem testes parciais. [2026-10-16] Roteiro tests/hw-smoke/integrated.sh escrito (13 passos, --preflight rodado no build PC); falta a execução com você presente. [2026-10-16 1º teste integrado] Primeira execução feita (passos 0-6 parcialmente); kextunload causou panic (HSCI em voo, corrigido F10 no código). Ver build-pc-runs/2026-10-16-first-integrated-run.md. [2026-10-17] R72: segundo Mac (MacBook Air via adaptador Thunderbolt-FireWire) funcionou com o pacote instalado.</t>
         </is>
       </c>
     </row>
@@ -27852,7 +27852,7 @@
       </c>
       <c r="I41" s="77" t="inlineStr">
         <is>
-          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: installer/build-pkg.sh. scripts/install.sh e uninstall.sh já funcionam no build PC (kext + daemon). [2026-10-17] R59: pacote .pkg não assinado montado no build PC (installer/make-pkg.sh): kext, helper+LaunchDaemon, painel, plug-in MIDI da referência, ícones, uninstall.sh; postinstall com portão kextutil -t -n. Instalado e atualizado no build PC (kext carrega de /Library/Extensions, helper roda, painel abre de /Applications, MIDI com ícone). Bug achado: bundles relocáveis/version-checked do pkgbuild (corrigido). Falta: máquina limpa, SIP ligado, aprovação do kext, reboot, teste do uninstall.sh. [2026-10-17] R69: imagem .dmg (instalador .pkg + app desinstalador, layout personalizado) via installer/make-dmg.sh; pkg com a correção de formato reinstalado no build PC; janela do desinstalador verificada; falta: botão Uninstall (senha de admin), máquina limpa, reboot, assinatura (IN.6).</t>
+          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: installer/build-pkg.sh. scripts/install.sh e uninstall.sh já funcionam no build PC (kext + daemon). [2026-10-17] R59: pacote .pkg não assinado montado no build PC (installer/make-pkg.sh): kext, helper+LaunchDaemon, painel, plug-in MIDI da referência, ícones, uninstall.sh; postinstall com portão kextutil -t -n. Instalado e atualizado no build PC (kext carrega de /Library/Extensions, helper roda, painel abre de /Applications, MIDI com ícone). Bug achado: bundles relocáveis/version-checked do pkgbuild (corrigido). Falta: máquina limpa, SIP ligado, aprovação do kext, reboot, teste do uninstall.sh. [2026-10-17] R69: imagem .dmg (instalador .pkg + app desinstalador, layout personalizado) via installer/make-dmg.sh; pkg com a correção de formato reinstalado no build PC; janela do desinstalador verificada; falta: botão Uninstall (senha de admin), máquina limpa, reboot, assinatura (IN.6). [2026-10-17] R72: imagem .dmg 0.1.0 reconstruída (runtime Swift embutido) instalada em um 2º Mac limpo (MacBook Air, 10.13.6, SIP desligado) via adaptador Thunderbolt-FireWire: instalou, reiniciou, driver carregou, painel abriu e funcionou (relato do usuário). Falta: SIP ligado / assinatura (IN.1, IN.6), botão Uninstall.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
README and installer text: homebrew, unsigned, requires SIP disabled; drop signing items
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PROVENANCE-MATRIX.xlsx
+++ b/PROVENANCE-MATRIX.xlsx
@@ -27649,7 +27649,7 @@
       </c>
       <c r="F37" s="77" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Cancelado (corte de escopo)</t>
         </is>
       </c>
       <c r="G37" s="77" t="inlineStr">
@@ -27664,7 +27664,7 @@
       </c>
       <c r="I37" s="77" t="inlineStr">
         <is>
-          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio.</t>
+          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-17] R73: decisão do usuário - projeto homebrew, sempre sem assinatura, exige SIP desligado; teste com SIP ligado fora do escopo.</t>
         </is>
       </c>
     </row>
@@ -27884,7 +27884,7 @@
       </c>
       <c r="F42" s="77" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Cancelado (corte de escopo)</t>
         </is>
       </c>
       <c r="G42" s="77" t="inlineStr">
@@ -27899,7 +27899,7 @@
       </c>
       <c r="I42" s="77" t="inlineStr">
         <is>
-          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: installer/sign.sh.</t>
+          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: installer/sign.sh. [2026-10-17] R73: decisão do usuário - sem assinatura Developer ID nem notarização, nunca.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
OpenAudio BeBoB MAFW 0.2.2: one driver for the FireWire 1814 and FireWire Audiophile
New tree openaudio-mafw-bebob/ (driver 0.2.0, panel OA BeBoB MAFW 1.3,
helper, installer that updates earlier versions in place), with the
FireWire Audiophile reverse-engineering notes and captures under docs/.
The 0.1.0 tree openaudio-fw1814/ is kept as released.
README: status, tested machines, known issues, repository map.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PROVENANCE-MATRIX.xlsx
+++ b/PROVENANCE-MATRIX.xlsx
@@ -26536,7 +26536,7 @@
       </c>
       <c r="I13" s="77" t="inlineStr">
         <is>
-          <t>[2026-10-15] Código escrito (R46/Q-MD2): FWSamples.{h,cpp}, FWDiscreteEngine clip/convert, FWBaseEngine::MainEngineClipOutputSamples/ConvertInputSamplesCore/ConvertInputSampleData, FWEngine2::ClipPCMOutput, FW1814Device::ResetRearrangementProcs/WorkaroundFor1814InputDelay, SetIOFormat chama ResetRearrangementProcs. Teste em host dos conversores OK; build PC limpo + kextutil -t -n OK; nada carregado. Não portado (fora do caminho do FW1814): _SamplePeaks*, LLRR, 1212CS, remap. Aceite (bytes idênticos ao oráculo, picos) só no teste integrado. [2026-10-15] Correção: o proc de peaks do FW1814 É usado (SwitchDigitalSignals) e foi portado no M-E (Q-ME §4).</t>
+          <t>[2026-10-15] Código escrito (R46/Q-MD2): FWSamples.{h,cpp}, FWDiscreteEngine clip/convert, FWBaseEngine::MainEngineClipOutputSamples/ConvertInputSamplesCore/ConvertInputSampleData, FWEngine2::ClipPCMOutput, FW1814Device::ResetRearrangementProcs/WorkaroundFor1814InputDelay, SetIOFormat chama ResetRearrangementProcs. Teste em host dos conversores OK; build PC limpo + kextutil -t -n OK; nada carregado. Não portado (fora do caminho do FW1814): _SamplePeaks*, LLRR, 1212CS, remap. Aceite (bytes idênticos ao oráculo, picos) só no teste integrado. [2026-10-15] Correção: o proc de peaks do FW1814 É usado (SwitchDigitalSignals) e foi portado no M-E (Q-ME §4). [2026-10-17] R75: performErase zeroed the sample buffer instead of the mix buffer (ref 0x4e08); fixed, loopcheck 34 s with 4 second-client events = 0 breaks; user confirmed by ear on the Air. Long soak NOT done.</t>
         </is>
       </c>
     </row>
@@ -26677,7 +26677,7 @@
       </c>
       <c r="I16" s="77" t="inlineStr">
         <is>
-          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: FWKIPCUserClient, FW1814UserClient. [2026-10-15] Código escrito (R48/Q-MF): FWKIPCUserClient, FW1814UserClient (seletores 500-507, memória, notificações tipo 0/1), entrega de propriedades. Build PC limpo + kextutil -t -n OK; nada carregado. Falta: MIDI real (M-H). Aceite só no teste integrado. [2026-10-16 1º teste integrado] User client, página de medidores e notificações funcionam com o painel real.</t>
+          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: FWKIPCUserClient, FW1814UserClient. [2026-10-15] Código escrito (R48/Q-MF): FWKIPCUserClient, FW1814UserClient (seletores 500-507, memória, notificações tipo 0/1), entrega de propriedades. Build PC limpo + kextutil -t -n OK; nada carregado. Falta: MIDI real (M-H). Aceite só no teste integrado. [2026-10-16 1º teste integrado] User client, página de medidores e notificações funcionam com o painel real. [2026-10-17] R76: performAudioEngineStop now calls ClearPeakMeters (ref 0x543c/0xda1e); user confirmed on the Air that the panel meters fall to zero after stop.</t>
         </is>
       </c>
     </row>
@@ -27476,7 +27476,7 @@
       </c>
       <c r="I33" s="77" t="inlineStr">
         <is>
-          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: control-panel/Sources/*.swift (AppDelegate, MaKeys, MixerView, MetersView, HardwareTab, IOKitBridge, Presets). Nada compilável ainda; wireframe (PN.1) é seu. [2026-10-16] Medidores: IOKitBridge (página compartilhada), peakToDB, mapa de slots, BusStrip/BusMeterPanel; janelas de mini medidores ainda não escritas. [2026-10-16] Janelas de mini medidores (largo/estreito) escritas e renderizadas em modo demo; slots de pico ainda sem teste com sinal real. [2026-10-16] Medidores LED com peak hold e clip; mini medidores agrupados (Analog/ADAT/S/PDIF), ADAT 5-8 acinzentados em 88.2/96. [2026-10-16 1º teste integrado] Medidores funcionando no hardware após F3.</t>
+          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: control-panel/Sources/*.swift (AppDelegate, MaKeys, MixerView, MetersView, HardwareTab, IOKitBridge, Presets). Nada compilável ainda; wireframe (PN.1) é seu. [2026-10-16] Medidores: IOKitBridge (página compartilhada), peakToDB, mapa de slots, BusStrip/BusMeterPanel; janelas de mini medidores ainda não escritas. [2026-10-16] Janelas de mini medidores (largo/estreito) escritas e renderizadas em modo demo; slots de pico ainda sem teste com sinal real. [2026-10-16] Medidores LED com peak hold e clip; mini medidores agrupados (Analog/ADAT/S/PDIF), ADAT 5-8 acinzentados em 88.2/96. [2026-10-16 1º teste integrado] Medidores funcionando no hardware após F3. [2026-10-17] R76: meters no longer freeze after audio stops (kext fix); verified by the user on the Air.</t>
         </is>
       </c>
     </row>
@@ -27852,7 +27852,7 @@
       </c>
       <c r="I41" s="77" t="inlineStr">
         <is>
-          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: installer/build-pkg.sh. scripts/install.sh e uninstall.sh já funcionam no build PC (kext + daemon). [2026-10-17] R59: pacote .pkg não assinado montado no build PC (installer/make-pkg.sh): kext, helper+LaunchDaemon, painel, plug-in MIDI da referência, ícones, uninstall.sh; postinstall com portão kextutil -t -n. Instalado e atualizado no build PC (kext carrega de /Library/Extensions, helper roda, painel abre de /Applications, MIDI com ícone). Bug achado: bundles relocáveis/version-checked do pkgbuild (corrigido). Falta: máquina limpa, SIP ligado, aprovação do kext, reboot, teste do uninstall.sh. [2026-10-17] R69: imagem .dmg (instalador .pkg + app desinstalador, layout personalizado) via installer/make-dmg.sh; pkg com a correção de formato reinstalado no build PC; janela do desinstalador verificada; falta: botão Uninstall (senha de admin), máquina limpa, reboot, assinatura (IN.6). [2026-10-17] R72: imagem .dmg 0.1.0 reconstruída (runtime Swift embutido) instalada em um 2º Mac limpo (MacBook Air, 10.13.6, SIP desligado) via adaptador Thunderbolt-FireWire: instalou, reiniciou, driver carregou, painel abriu e funcionou (relato do usuário). Falta: SIP ligado / assinatura (IN.1, IN.6), botão Uninstall.</t>
+          <t>[2026-10-15] G1 aprovado pelo usuário; construção segue o fluxograma docs/flowchart driver.drawio. [2026-10-15] Esqueleto: installer/build-pkg.sh. scripts/install.sh e uninstall.sh já funcionam no build PC (kext + daemon). [2026-10-17] R59: pacote .pkg não assinado montado no build PC (installer/make-pkg.sh): kext, helper+LaunchDaemon, painel, plug-in MIDI da referência, ícones, uninstall.sh; postinstall com portão kextutil -t -n. Instalado e atualizado no build PC (kext carrega de /Library/Extensions, helper roda, painel abre de /Applications, MIDI com ícone). Bug achado: bundles relocáveis/version-checked do pkgbuild (corrigido). Falta: máquina limpa, SIP ligado, aprovação do kext, reboot, teste do uninstall.sh. [2026-10-17] R69: imagem .dmg (instalador .pkg + app desinstalador, layout personalizado) via installer/make-dmg.sh; pkg com a correção de formato reinstalado no build PC; janela do desinstalador verificada; falta: botão Uninstall (senha de admin), máquina limpa, reboot, assinatura (IN.6). [2026-10-17] R72: imagem .dmg 0.1.0 reconstruída (runtime Swift embutido) instalada em um 2º Mac limpo (MacBook Air, 10.13.6, SIP desligado) via adaptador Thunderbolt-FireWire: instalou, reiniciou, driver carregou, painel abriu e funcionou (relato do usuário). Falta: SIP ligado / assinatura (IN.1, IN.6), botão Uninstall. [2026-10-17] 2026-10-17 pkg+dmg rebuilt with R75+R76 (kext FC8AD9DA), sha256 dmg 473dce40...3422, self-contained checks passed; not installed from this image yet; release asset to be replaced by the user.</t>
         </is>
       </c>
     </row>

</xml_diff>